<commit_message>
fix(shell): keep a destination whole when the fallback copy fails, and stop guessing table ownership
</commit_message>
<xml_diff>
--- a/e2e/atago/testdata/sheets_names.xlsx
+++ b/e2e/atago/testdata/sheets_names.xlsx
@@ -10,11 +10,10 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="a-b-c" sheetId="2" r:id="rId4"/>
     <sheet name="a  b" sheetId="3" r:id="rId6"/>
-    <sheet name="a..b" sheetId="4" r:id="rId7"/>
-    <sheet name="x(1)" sheetId="5" r:id="rId8"/>
-    <sheet name="Ünïcode" sheetId="6" r:id="rId9"/>
-    <sheet name="  pad  " sheetId="7" r:id="rId10"/>
-    <sheet name="table" sheetId="8" r:id="rId11"/>
+    <sheet name="x(1)" sheetId="4" r:id="rId7"/>
+    <sheet name="Ünïcode" sheetId="5" r:id="rId8"/>
+    <sheet name="  pad  " sheetId="6" r:id="rId9"/>
+    <sheet name="table" sheetId="7" r:id="rId10"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
@@ -453,22 +452,4 @@
     </row>
   </sheetData>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-</worksheet>
 </file>
</xml_diff>